<commit_message>
feat: extract invoice numbers from boletos and include them in the NFSe generation payload
</commit_message>
<xml_diff>
--- a/upload/EXCEL/Template_VR.xlsx
+++ b/upload/EXCEL/Template_VR.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Importacao_Completa" sheetId="1" state="visible" r:id="rId3"/>
@@ -620,11 +620,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1040,7 +1040,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="90.22"/>
@@ -1514,7 +1514,6 @@
       <c r="D46" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="E46" s="0"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
@@ -1570,7 +1569,6 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0"/>
       <c r="B51" s="15" t="s">
         <v>120</v>
       </c>
@@ -1591,36 +1589,6 @@
       <c r="D52" s="15" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="0"/>
-      <c r="C53" s="0"/>
-      <c r="D53" s="0"/>
-    </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="0"/>
-      <c r="C54" s="0"/>
-      <c r="D54" s="0"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="0"/>
-      <c r="C55" s="0"/>
-      <c r="D55" s="0"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="0"/>
-      <c r="C56" s="0"/>
-      <c r="D56" s="0"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="0"/>
-      <c r="C57" s="0"/>
-      <c r="D57" s="0"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="0"/>
-      <c r="C58" s="0"/>
-      <c r="D58" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
update: refresh import templates with latest schema changes
</commit_message>
<xml_diff>
--- a/upload/EXCEL/Template_VR.xlsx
+++ b/upload/EXCEL/Template_VR.xlsx
@@ -11,9 +11,6 @@
     <sheet name="Importacao_Completa" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Instruções" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Importacao_Completa!$A$1:$Z$1</definedName>
-  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -24,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="124">
-  <si>
-    <t xml:space="preserve">cnpj_condominio*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_condominio*</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="117">
+  <si>
+    <t xml:space="preserve">cnpj_condominio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_condominio</t>
   </si>
   <si>
     <t xml:space="preserve">tipo_local_condominio</t>
@@ -56,13 +53,13 @@
     <t xml:space="preserve">cep_condominio</t>
   </si>
   <si>
-    <t xml:space="preserve">cpf_funcionario*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matricula_funcionario*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_funcionario*</t>
+    <t xml:space="preserve">cpf_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matricula_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcionario</t>
   </si>
   <si>
     <t xml:space="preserve">funcao_funcionario</t>
@@ -95,10 +92,10 @@
     <t xml:space="preserve">nome_produto</t>
   </si>
   <si>
-    <t xml:space="preserve">data_competencia*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valor_beneficio(total)*</t>
+    <t xml:space="preserve">data_competencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_beneficio(total)</t>
   </si>
   <si>
     <t xml:space="preserve">quantidade_dias</t>
@@ -155,9 +152,6 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">cnpj_condominio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sim *</t>
   </si>
   <si>
@@ -167,9 +161,6 @@
     <t xml:space="preserve">B</t>
   </si>
   <si>
-    <t xml:space="preserve">nome_condominio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome/Razão social do condomínio</t>
   </si>
   <si>
@@ -227,27 +218,18 @@
     <t xml:space="preserve">K</t>
   </si>
   <si>
-    <t xml:space="preserve">cpf_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">CPF do funcionário (apenas números, 11 dígitos)</t>
   </si>
   <si>
     <t xml:space="preserve">L</t>
   </si>
   <si>
-    <t xml:space="preserve">matricula_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">Matrícula do funcionário</t>
   </si>
   <si>
     <t xml:space="preserve">M</t>
   </si>
   <si>
-    <t xml:space="preserve">nome_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome completo do funcionário</t>
   </si>
   <si>
@@ -314,16 +296,10 @@
     <t xml:space="preserve">X</t>
   </si>
   <si>
-    <t xml:space="preserve">data_competencia</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data de competência (dd/mm/aaaa)</t>
   </si>
   <si>
     <t xml:space="preserve">Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valor_beneficio(total)</t>
   </si>
   <si>
     <t xml:space="preserve">Valor total do benefício em R$</t>
@@ -637,32 +613,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -724,10 +674,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -910,36 +856,36 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z1048576"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="29.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="19.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="25.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="22.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="22.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="31.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="20.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="28.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="32.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="38.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="31.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="2" width="19.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="18.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="3" width="22.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="4" width="25.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="19.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="27" style="1" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="21.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="18.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="24.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="37.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="29.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="31.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="36.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="29.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="2" width="17.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="17.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="3" width="21.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="4" width="24.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="18.68"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="27" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1022,8 +968,41 @@
         <v>25</v>
       </c>
     </row>
+    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:Z1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1031,7 +1010,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1132,462 +1110,462 @@
         <v>42</v>
       </c>
       <c r="B17" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="D17" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>46</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>2</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>5</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>18</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>19</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B39" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>99</v>
+        <v>24</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B42" s="12" t="s">
         <v>25</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C47" s="15" t="n">
         <v>204</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C48" s="15" t="n">
         <v>207</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C49" s="15" t="n">
         <v>27</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="15" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C50" s="15" t="n">
         <v>28</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="15" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C51" s="15" t="n">
         <v>201</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="15" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C52" s="15" t="n">
         <v>202</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>